<commit_message>
feat: ensure single date selection generates exactly 1 specific day schedule
</commit_message>
<xml_diff>
--- a/Template_Import_Jadwal_Roster.xlsx
+++ b/Template_Import_Jadwal_Roster.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="17">
   <si>
     <t>nik</t>
   </si>
@@ -23,7 +23,10 @@
     <t>nama_karyawan</t>
   </si>
   <si>
-    <t>tanggal</t>
+    <t>tanggal_mulai</t>
+  </si>
+  <si>
+    <t>tanggal_akhir</t>
   </si>
   <si>
     <t>shift</t>
@@ -32,13 +35,16 @@
     <t>lokasi_kerja</t>
   </si>
   <si>
-    <t>tipe_jadwal</t>
+    <t>3571010904890004</t>
   </si>
   <si>
     <t>ZAIN AZIIZ</t>
   </si>
   <si>
-    <t>2026-08-20</t>
+    <t>2026-08-01</t>
+  </si>
+  <si>
+    <t>2026-08-31</t>
   </si>
   <si>
     <t>OFFICE</t>
@@ -47,22 +53,19 @@
     <t>INHOUSE AMK SURABAYA</t>
   </si>
   <si>
-    <t>workday</t>
-  </si>
-  <si>
-    <t>2026-08-21</t>
+    <t>3671084906990003</t>
   </si>
   <si>
     <t xml:space="preserve">Nitta Tridadi </t>
   </si>
   <si>
+    <t>3513174403000002</t>
+  </si>
+  <si>
     <t>Warda</t>
   </si>
   <si>
     <t>OFF</t>
-  </si>
-  <si>
-    <t>dayoff</t>
   </si>
 </sst>
 </file>
@@ -99,7 +102,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4F46E5"/>
+        <fgColor rgb="FF1E3A8A"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -116,8 +119,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="49" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="49" fillId="2" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -418,155 +423,95 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="19.995" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="19.995" bestFit="true" customWidth="true" style="1"/>
     <col min="2" max="2" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="8.141" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="24.708" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2">
-        <v>3571010904890004</v>
+      <c r="A2" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3">
-        <v>3571010904890004</v>
+      <c r="A3" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
         <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4">
-        <v>3671084906990003</v>
+      <c r="A4" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5">
-        <v>3671084906990003</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
         <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6">
-        <v>3513174403000002</v>
-      </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7">
-        <v>3513174403000002</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F7" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enhance date parser in schedule import to seamlessly handle d/m/Y (e.g. 21/08/2026)
</commit_message>
<xml_diff>
--- a/Template_Import_Jadwal_Roster.xlsx
+++ b/Template_Import_Jadwal_Roster.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My File\Project APlikasi Absensi\New\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4FCCE01-7964-430A-82AF-8CD1D732181F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <calcPr calcId="191029" forceFullCalc="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>nik</t>
   </si>
@@ -35,59 +40,30 @@
     <t>lokasi_kerja</t>
   </si>
   <si>
-    <t>3571010904890004</t>
-  </si>
-  <si>
-    <t>ZAIN AZIIZ</t>
-  </si>
-  <si>
-    <t>2026-08-01</t>
-  </si>
-  <si>
-    <t>2026-08-31</t>
-  </si>
-  <si>
     <t>OFFICE</t>
   </si>
   <si>
     <t>INHOUSE AMK SURABAYA</t>
   </si>
   <si>
-    <t>3671084906990003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nitta Tridadi </t>
-  </si>
-  <si>
-    <t>3513174403000002</t>
-  </si>
-  <si>
-    <t>Warda</t>
-  </si>
-  <si>
-    <t>OFF</t>
+    <t>3528042504850003</t>
+  </si>
+  <si>
+    <t>ABDURRAHMAN JAMIL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
@@ -119,17 +95,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="49" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="49" fillId="2" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -419,22 +405,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.995" bestFit="true" customWidth="true" style="1"/>
-    <col min="2" max="2" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="24.708" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -454,78 +436,27 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="5">
+        <v>46255</v>
+      </c>
+      <c r="D2" s="5">
+        <v>46285</v>
+      </c>
+      <c r="E2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="F2" t="s">
         <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: transform itineraries into Visit Schedule with Calendar view, checkin location marker, and Excel import
</commit_message>
<xml_diff>
--- a/Template_Import_Jadwal_Roster.xlsx
+++ b/Template_Import_Jadwal_Roster.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My File\Project APlikasi Absensi\New\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10452FD8-1087-4221-8466-4E7B3EA05EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE39CC0E-3FBB-4917-A937-9163D7A5C7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -444,7 +444,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="5">
-        <v>46255</v>
+        <v>46224</v>
       </c>
       <c r="D2" s="5">
         <v>46285</v>

</xml_diff>